<commit_message>
Corregir redacción del caso parcial de recubrimiento: "gran parte" en vez de "un tramo"
El usuario señaló que un tramo puntual/aislado no se pinta -- el
mantenimiento de recubrimiento siempre cubre la totalidad del circuito o
una gran parte de él (por eso se registra la longitud aproximada). El
caso TUBERIA_DETERIORO_RECUBRIMIENTO_PARCIAL decía "en un tramo de NPS
X", dando a entender un punto aislado; ahora dice "en gran parte del
recubrimiento (pintura) del circuito NPS X (longitud aprox. Y metros)",
conservando la longitud como justificación de esa extensión parcial (a
diferencia del caso GENERALIZADO, que cubre la totalidad y no necesita
mencionar longitud).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cu3g7hFxThiRvabaVjDM4F
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -773,12 +773,12 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Deterioro del recubrimiento y corrosión leve a moderada en {elemento} (tramo NPS {nps}, longitud aprox. {longitud} metros).</t>
+          <t>Deterioro del recubrimiento y corrosión leve a moderada en {elemento} (circuito NPS {nps}, longitud aprox. {longitud} metros).</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Efectuar el mantenimiento del recubrimiento (pintura) en un tramo de NPS {nps}, siguiendo los estándares Repsol ED-B-06.00-04d y el documento PE-B-0600.01H00R05.</t>
+          <t>Efectuar el mantenimiento en gran parte del recubrimiento (pintura) del circuito NPS {nps} (longitud aprox. {longitud} metros), siguiendo los estándares Repsol ED-B-06.00-04d y el documento PE-B-0600.01H00R05.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Mencionar cantidad de tramos en la recomendación de recubrimiento parcial
Cuando el mantenimiento cubre "gran parte" del circuito (caso
TUBERIA_DETERIORO_RECUBRIMIENTO_PARCIAL) ahora se indica en cuántos
tramos, tomando la cantidad del propio hallazgo de campo (mismo
mecanismo de extracción y de resolución singular/plural "tramo(s)" que
ya usa el resto del catálogo, p.ej. "válvula(s)"): "en 1 tramo" o "en 2
tramos" según corresponda. Si el hallazgo no especifica cantidad, se usa
el valor por defecto (1). El caso de circuito completo (GENERALIZADO)
no se toca -- sigue sin mencionar tramo, porque cubre la totalidad.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cu3g7hFxThiRvabaVjDM4F
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -778,17 +778,17 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Efectuar el mantenimiento en gran parte del recubrimiento (pintura) del circuito NPS {nps} (longitud aprox. {longitud} metros), siguiendo los estándares Repsol ED-B-06.00-04d y el documento PE-B-0600.01H00R05.</t>
+          <t>Efectuar el mantenimiento en gran parte del recubrimiento (pintura) del circuito NPS {nps}, en {cantidad} tramo(s) (longitud aprox. {longitud} metros), siguiendo los estándares Repsol ED-B-06.00-04d y el documento PE-B-0600.01H00R05.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>elemento, nps, longitud</t>
+          <t>elemento, nps, longitud, cantidad</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>elemento=los accesorios y componentes</t>
+          <t>elemento=los accesorios y componentes; cantidad=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Habilita las reglas de bridas también bajo el ítem "Placas orificio"
Bug real reportado por el usuario: un hallazgo de espárragos cortos en
la brida de una placa orificio quedó PENDIENTE, aunque el caso
BRIDA_ESPARRAGOS_CORTOS ya tenía regla (agregada en el commit
anterior). Causa: las placas orificio tienen sus propias bridas con
espárragos, y el inspector anotó el hallazgo bajo el ítem "Placas
orificio" del checklist (no bajo "Bridas..."), pero todas las reglas
de bridas -- las 7 que ya existían y las 4 agregadas hoy -- solo
estaban habilitadas para la categoría "bridas", nunca para "placas
orificio".

Se amplía la categoría de las 11 reglas de bridas a
"bridas; placas orificio". Verificado: los 10 casos BRIDA/BRIDA_ORIFICIO
del catálogo se auto-sugieren correctamente tanto bajo "Bridas..." como
bajo "Placas orificio", sin ninguna colisión nueva.
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D4" s="7" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D6" s="7" t="n">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D54" s="6" t="n">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D56" s="6" t="n">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D97" t="n">

</xml_diff>

<commit_message>
Habilita las reglas de bridas también bajo el ítem "Placas orificio" (#46)
Bug real reportado por el usuario: un hallazgo de espárragos cortos en
la brida de una placa orificio quedó PENDIENTE, aunque el caso
BRIDA_ESPARRAGOS_CORTOS ya tenía regla (agregada en el commit
anterior). Causa: las placas orificio tienen sus propias bridas con
espárragos, y el inspector anotó el hallazgo bajo el ítem "Placas
orificio" del checklist (no bajo "Bridas..."), pero todas las reglas
de bridas -- las 7 que ya existían y las 4 agregadas hoy -- solo
estaban habilitadas para la categoría "bridas", nunca para "placas
orificio".

Se amplía la categoría de las 11 reglas de bridas a
"bridas; placas orificio". Verificado: los 10 casos BRIDA/BRIDA_ORIFICIO
del catálogo se auto-sugieren correctamente tanto bajo "Bridas..." como
bajo "Placas orificio", sin ninguna colisión nueva.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D4" s="7" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D6" s="7" t="n">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D54" s="6" t="n">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D56" s="6" t="n">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>bridas</t>
+          <t>bridas; placas orificio</t>
         </is>
       </c>
       <c r="D97" t="n">

</xml_diff>

<commit_message>
Ajustar TUBERIA_TRAMO_NO_ACCESIBLE a la redaccion literal del compendio
El caso de "tramo no accesible / en altura" ya existia, pero parafraseaba
en vez de usar la frase que exige el compendio para este hallazgo
("presencia de corrosion (otros) en tramo no accesible") -- se corrige
por fidelidad literal, mismo criterio ya aplicado al resto del catalogo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cu3g7hFxThiRvabaVjDM4F
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -881,12 +881,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Circuito NPS {nps} evidencia corrosión en zonas sin acceso para inspección visual adecuada, por encontrarse en altura.</t>
+          <t>Presencia de corrosión (otros) en tramo no accesible de la línea NPS {nps}, cerca de {ubicacion}, por encontrarse en altura, lo que no permite calificar su severidad mediante inspección visual (VT).</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Se requiere instalar facilidades (andamios de {longitud} metros) para acceder a la zona cerca de {ubicacion} y complementar la inspección de la zona observada en la tubería de NPS {nps}.</t>
+          <t>Instalar facilidades de acceso (andamios de {longitud} metros) cerca de {ubicacion} para realizar la inspección visual (VT) adecuada de la línea NPS {nps} y determinar el grado de corrosión (daño) real.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Capturar la separacion medida en desviacion de paralelismo de brida
BRIDA_MONTAJE_PARALELISMO_INCORRECTO ya existia (misma recomendacion
que pidio el usuario), pero su hallazgo_tpl era generico y no
reflejaba la separacion medida (p.ej. "de 6 mm a 8 mm") que el
inspector sí registra en campo -- se agrega la variable {separacion},
su extraccion por regex (RE_SEPARACION_MM, admite rango o valor unico)
y el patron de omision correspondiente para el peor caso (sin dato).

Verificado con el texto real del hallazgo proporcionado por el
usuario (auto-match exacto) y la regresion completa del catalogo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cu3g7hFxThiRvabaVjDM4F
</commit_message>
<xml_diff>
--- a/Catalogo_Hallazgos_Recomendaciones.xlsx
+++ b/Catalogo_Hallazgos_Recomendaciones.xlsx
@@ -2653,7 +2653,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Se evidencia falta de paralelismo en el montaje de la unión bridada de NPS {nps}.</t>
+          <t>Desviación de paralelismo entre caras de brida en unión bridada de NPS {nps}, con una separación de {separacion}.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>nps</t>
+          <t>nps, separacion</t>
         </is>
       </c>
     </row>

</xml_diff>